<commit_message>
fixed unit conversion bugs
</commit_message>
<xml_diff>
--- a/config_data/units_mapping_pow.xlsx
+++ b/config_data/units_mapping_pow.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>EUR/(MW*a)</t>
   </si>
@@ -540,9 +540,7 @@
       <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>8</v>
-      </c>
+      <c r="B11" s="3"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -554,9 +552,6 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance emission factor processing by adding unit conversion and error logging; update units mapping and ignore prefixes for improved data handling
</commit_message>
<xml_diff>
--- a/config_data/units_mapping_pow.xlsx
+++ b/config_data/units_mapping_pow.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>EUR/(MW*a)</t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>Desired_Unit</t>
+  </si>
+  <si>
+    <t>g/GJ</t>
   </si>
 </sst>
 </file>
@@ -452,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
@@ -563,10 +566,19 @@
         <v>18</v>
       </c>
     </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+    </row>
   </sheetData>
   <sortState ref="A2:B14">
     <sortCondition ref="A1"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>